<commit_message>
Gem mine valg (sport + danske backdrops) 2026-10-05 23:09:46
</commit_message>
<xml_diff>
--- a/data/danish_artwork_review.xlsx
+++ b/data/danish_artwork_review.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EPGoal\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2257F572-88AF-4F5B-A5CF-1AB6D85636EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BA6FC9F-A7EA-4529-9C8B-F1ACD119A5B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danske backdrops" sheetId="1" r:id="rId1"/>

</xml_diff>